<commit_message>
Adding all trade links
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Trades/ScenTrade__Trade_Links.xlsx
+++ b/VerveStacks_EST/SuppXLS/Trades/ScenTrade__Trade_Links.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\Trades\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A70F9AE-22CD-46B5-B61A-DC8978A30DD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3E6B7F-1101-4A3B-99B5-0996A850F7EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BI" sheetId="5" r:id="rId1"/>
@@ -331,13 +331,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -945,7 +944,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3:O27"/>
+  <dimension ref="C3:M23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -956,656 +955,592 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C3" s="5" t="s">
+      <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5" t="s">
+      <c r="L3" t="s">
         <v>5</v>
       </c>
-      <c r="M3" s="5"/>
     </row>
     <row r="4" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C4" s="5" t="s">
+      <c r="C4" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5" t="s">
+      <c r="L4" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="M4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" t="s">
         <v>32</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5" t="s">
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" t="s">
         <v>32</v>
       </c>
-      <c r="M5" s="5" t="s">
+      <c r="M5" t="s">
         <v>51</v>
       </c>
     </row>
+    <row r="6" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7" t="s">
+        <v>34</v>
+      </c>
+      <c r="M7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+      <c r="L8" t="s">
+        <v>35</v>
+      </c>
+      <c r="M8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" t="s">
+        <v>36</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+      <c r="L9" t="s">
+        <v>36</v>
+      </c>
+      <c r="M9" t="s">
+        <v>55</v>
+      </c>
+    </row>
     <row r="10" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C10" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" s="5" t="s">
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" t="s">
+        <v>37</v>
+      </c>
+      <c r="M10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" t="s">
         <v>19</v>
       </c>
-      <c r="H10" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C11" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>53</v>
+      <c r="H11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+      <c r="L11" t="s">
+        <v>38</v>
+      </c>
+      <c r="M11" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C12" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="5" t="s">
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" t="s">
+        <v>39</v>
+      </c>
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+      <c r="L12" t="s">
+        <v>39</v>
+      </c>
+      <c r="M12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" t="s">
+        <v>40</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+      <c r="L13" t="s">
+        <v>40</v>
+      </c>
+      <c r="M13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" t="s">
         <v>21</v>
       </c>
-      <c r="H12" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="M12" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="13" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="5" t="s">
+      <c r="H14" t="s">
+        <v>41</v>
+      </c>
+      <c r="I14" t="s">
+        <v>16</v>
+      </c>
+      <c r="L14" t="s">
+        <v>41</v>
+      </c>
+      <c r="M14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" t="s">
+        <v>29</v>
+      </c>
+      <c r="H15" t="s">
+        <v>42</v>
+      </c>
+      <c r="I15" t="s">
+        <v>16</v>
+      </c>
+      <c r="L15" t="s">
+        <v>42</v>
+      </c>
+      <c r="M15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" t="s">
+        <v>23</v>
+      </c>
+      <c r="H16" t="s">
+        <v>43</v>
+      </c>
+      <c r="I16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L16" t="s">
+        <v>43</v>
+      </c>
+      <c r="M16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H17" t="s">
+        <v>44</v>
+      </c>
+      <c r="I17" t="s">
+        <v>16</v>
+      </c>
+      <c r="L17" t="s">
+        <v>44</v>
+      </c>
+      <c r="M17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G18" t="s">
+        <v>23</v>
+      </c>
+      <c r="H18" t="s">
+        <v>45</v>
+      </c>
+      <c r="I18" t="s">
+        <v>16</v>
+      </c>
+      <c r="L18" t="s">
+        <v>45</v>
+      </c>
+      <c r="M18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M13" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="14" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C14" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F14" s="5" t="s">
+      <c r="G19" t="s">
+        <v>26</v>
+      </c>
+      <c r="H19" t="s">
+        <v>46</v>
+      </c>
+      <c r="I19" t="s">
+        <v>16</v>
+      </c>
+      <c r="L19" t="s">
+        <v>46</v>
+      </c>
+      <c r="M19" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="M14" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="15" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C15" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="M15" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C16" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="M16" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="17" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C17" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="M17" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="18" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C18" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F18" s="5" t="s">
+      <c r="G20" t="s">
+        <v>22</v>
+      </c>
+      <c r="H20" t="s">
+        <v>47</v>
+      </c>
+      <c r="I20" t="s">
+        <v>16</v>
+      </c>
+      <c r="L20" t="s">
+        <v>47</v>
+      </c>
+      <c r="M20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21" t="s">
+        <v>30</v>
+      </c>
+      <c r="G21" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" t="s">
+        <v>48</v>
+      </c>
+      <c r="I21" t="s">
+        <v>16</v>
+      </c>
+      <c r="L21" t="s">
+        <v>48</v>
+      </c>
+      <c r="M21" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" t="s">
         <v>27</v>
       </c>
-      <c r="G18" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="M18" t="s">
-        <v>59</v>
-      </c>
-      <c r="O18" s="5"/>
-    </row>
-    <row r="19" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C19" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="M19" t="s">
-        <v>60</v>
-      </c>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-    </row>
-    <row r="20" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="M20" t="s">
-        <v>61</v>
-      </c>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-    </row>
-    <row r="21" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C21" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="M21" t="s">
-        <v>62</v>
-      </c>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-    </row>
-    <row r="22" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C22" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="I22" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5" t="s">
-        <v>45</v>
+      <c r="G22" t="s">
+        <v>31</v>
+      </c>
+      <c r="H22" t="s">
+        <v>49</v>
+      </c>
+      <c r="I22" t="s">
+        <v>16</v>
+      </c>
+      <c r="L22" t="s">
+        <v>49</v>
       </c>
       <c r="M22" t="s">
-        <v>63</v>
-      </c>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-    </row>
-    <row r="23" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C23" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F23" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F23" t="s">
+        <v>31</v>
+      </c>
+      <c r="G23" t="s">
         <v>22</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5" t="s">
-        <v>46</v>
+      <c r="H23" t="s">
+        <v>50</v>
+      </c>
+      <c r="I23" t="s">
+        <v>16</v>
+      </c>
+      <c r="L23" t="s">
+        <v>50</v>
       </c>
       <c r="M23" t="s">
-        <v>64</v>
-      </c>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-    </row>
-    <row r="24" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C24" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="I24" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M24" t="s">
-        <v>65</v>
-      </c>
-      <c r="N24" s="5"/>
-      <c r="O24" s="5"/>
-    </row>
-    <row r="25" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C25" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="I25" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="M25" t="s">
-        <v>66</v>
-      </c>
-      <c r="N25" s="5"/>
-      <c r="O25" s="5"/>
-    </row>
-    <row r="26" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C26" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="L26" t="s">
-        <v>49</v>
-      </c>
-      <c r="M26" t="s">
-        <v>67</v>
-      </c>
-      <c r="N26" s="5"/>
-      <c r="O26" s="5"/>
-    </row>
-    <row r="27" spans="3:15" x14ac:dyDescent="0.25">
-      <c r="C27" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="L27" t="s">
-        <v>50</v>
-      </c>
-      <c r="M27" t="s">
         <v>68</v>
       </c>
-      <c r="N27" s="5"/>
-      <c r="O27" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>